<commit_message>
feat: Update estado_del_arte.xlsx with new findings and sources
</commit_message>
<xml_diff>
--- a/estado_del_arte.xlsx
+++ b/estado_del_arte.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentación INDEC" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Estado del arte'!$A$1:$K$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Estado del arte'!$A$1:$K$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Documentación INDEC'!$A$1:$E$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -68,7 +68,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -119,6 +119,21 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -139,7 +154,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -181,6 +196,15 @@
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -485,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="5" min="1" max="1"/>
@@ -2525,8 +2549,888 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>Albina, I., Gasparini, L., Tornarolli, L.</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>Medición de la pobreza en contextos de inflación cambiante: el caso de Argentina (CEDLAS WP Nº 370)</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>Cuantificar cómo la medición de la pobreza por ingresos se ve afectada por aspectos metodológicos en alta inflación: desfasaje EPH-canasta, subreporte de ingresos, y reestimación del Coeficiente de Engel con ENGH 2017/18.</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>Comparación EPH vs registros administrativos + reestimación Engel con ENGH 2017/18; período 2018-2025.</t>
+        </is>
+      </c>
+      <c r="H40" s="15" t="inlineStr">
+        <is>
+          <t>Las tres correcciones tienen efectos cuantitativamente relevantes sobre el nivel y la evolución de la tasa de pobreza. Marco replicable.</t>
+        </is>
+      </c>
+      <c r="I40" s="15" t="inlineStr">
+        <is>
+          <t>ESPEJO ARGENTINO DIRECTO post-pivote Rosati. Mismo período, misma encuesta de gasto, misma universidad. Cita central de motivación + validación del recorte 2017+.</t>
+        </is>
+      </c>
+      <c r="J40" s="15" t="inlineStr">
+        <is>
+          <t>https://www.cedlas.econo.unlp.edu.ar/wp/wp-content/uploads/doc_cedlas370.pdf</t>
+        </is>
+      </c>
+      <c r="K40" s="15" t="inlineStr">
+        <is>
+          <t>TP — must-have ⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>Albina, I., Laguinge, L., Gasparini, L., Tornarolli, L., Cruces, G., Afonso, S.</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>Ajustando la Imagen de la Distribución del Ingreso en Argentina: Encuestas y Registros Administrativos (CEDLAS WP Nº 336)</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>Estimar la distribución del ingreso en Argentina combinando microdatos de la EPH con registros administrativos (salarios formales, monotributo, autónomos, ganancias, jubilaciones, transferencias).</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>Combinación EPH + registros administrativos.</t>
+        </is>
+      </c>
+      <c r="H41" s="15" t="inlineStr">
+        <is>
+          <t>Las correcciones por subreporte y registros administrativos cambian sustancialmente la imagen de la distribución del ingreso en Argentina.</t>
+        </is>
+      </c>
+      <c r="I41" s="15" t="inlineStr">
+        <is>
+          <t>Antecedente local del tratamiento de ingresos EPH. Útil para discutir el problema del subreporte en la EPH continua del proyecto.</t>
+        </is>
+      </c>
+      <c r="J41" s="15" t="inlineStr">
+        <is>
+          <t>https://www.cedlas.econo.unlp.edu.ar/wp/wp-content/uploads/doc_cedlas336.pdf</t>
+        </is>
+      </c>
+      <c r="K41" s="15" t="inlineStr">
+        <is>
+          <t>TP — must-have ⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>Argente, D., Lee, M.</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>Cost of Living Inequality during the Great Recession</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>Construir índices de precios por cuartil de ingreso para EE.UU. 2004-2016 y medir el gap de inflación durante la Gran Recesión.</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>Índices Laspeyres por cuartil con scanner data + CES; descomposición por sustitución de calidad y comportamiento de compra.</t>
+        </is>
+      </c>
+      <c r="H42" s="15" t="inlineStr">
+        <is>
+          <t>El cuartil más pobre experimentó inflación 2.4x mayor que el más rico durante 2008-2013. ~40% del gap se explica por sustitución de calidad y cambios en comportamiento de compra (más accesibles a los ricos).</t>
+        </is>
+      </c>
+      <c r="I42" s="15" t="inlineStr">
+        <is>
+          <t>Espejo metodológico canónico de IPC distribuido durante recesiones. Replica conceptual lo que Argentina vivió 2018-2024.</t>
+        </is>
+      </c>
+      <c r="J42" s="15" t="inlineStr">
+        <is>
+          <t>https://academic.oup.com/jeea/article-abstract/19/2/913/5863149</t>
+        </is>
+      </c>
+      <c r="K42" s="15" t="inlineStr">
+        <is>
+          <t>TP — must-have ⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>Kaplan, G., Schulhofer-Wohl, S.</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>Inflation at the Household Level</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>Medir y descomponer la heterogeneidad de inflación a nivel hogar en EE.UU. usando scanner data.</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>IPC a nivel hogar usando scanner data + CES; descomposición de la varianza entre canastas vs precios pagados por bienes idénticos.</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="inlineStr">
+        <is>
+          <t>IQR de la inflación entre hogares: 6.2-9.0 pp anual. CRÍTICO: solo ~7% de la varianza se explica por diferencias en canastas; ~2/3 viene de precios pagados por bienes idénticos y ~1/3 de variedad dentro de categorías.</t>
+        </is>
+      </c>
+      <c r="I43" s="15" t="inlineStr">
+        <is>
+          <t>ADVERTENCIA estructural al proyecto: si Kaplan-Schulhofer-Wohl tienen razón, la heterogeneidad de canastas explica solo ~7% de la inflación heterogénea total. Hay que declararlo como limitación o argumentar por qué Argentina puede ser distinta.</t>
+        </is>
+      </c>
+      <c r="J43" s="15" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jmoneco.2017.08.002</t>
+        </is>
+      </c>
+      <c r="K43" s="15" t="inlineStr">
+        <is>
+          <t>TP — must-have ⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>Cravino, J., Lan, T., Levchenko, A.</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>Price Stickiness Along the Income Distribution and the Effects of Monetary Policy</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>Estudiar cómo la rigidez de precios varía a lo largo de la distribución del ingreso y sus consecuencias para política monetaria.</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="inlineStr">
+        <is>
+          <t>Análisis empírico de stickiness por categoría de gasto + impulso-respuesta a shocks monetarios.</t>
+        </is>
+      </c>
+      <c r="H44" s="15" t="inlineStr">
+        <is>
+          <t>Los precios de bienes consumidos por hogares de altos ingresos son más rígidos. Tras un shock monetario, las respuestas del IPC de altos ingresos son ~1/3 menores que las de ingresos medios.</t>
+        </is>
+      </c>
+      <c r="I44" s="15" t="inlineStr">
+        <is>
+          <t>Marco teórico: la heterogeneidad de canastas tiene consecuencias macroeconómicas (no solo distributivas). Refuerza la motivación.</t>
+        </is>
+      </c>
+      <c r="J44" s="15" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jmoneco.2019.10.003</t>
+        </is>
+      </c>
+      <c r="K44" s="15" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>Cravino, J., Levchenko, A.</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>The Distributional Consequences of Large Devaluations</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>Estudiar cómo las grandes devaluaciones del tipo de cambio afectan diferencialmente a hogares según ingreso.</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="inlineStr">
+        <is>
+          <t>Análisis empírico de elasticidades de gasto + cambios en precios relativos durante crisis cambiarias.</t>
+        </is>
+      </c>
+      <c r="H45" s="15" t="inlineStr">
+        <is>
+          <t>Los hogares pobres gastan más en bienes transables y variedades baratas, sufriendo mayor inflación durante devaluaciones.</t>
+        </is>
+      </c>
+      <c r="I45" s="15" t="inlineStr">
+        <is>
+          <t>Particularmente relevante para Argentina (devaluaciones recurrentes). Cita en la motivación del impacto distributivo de la inflación argentina.</t>
+        </is>
+      </c>
+      <c r="J45" s="15" t="inlineStr">
+        <is>
+          <t>https://www.aeaweb.org/articles?id=10.1257/aer.20151551</t>
+        </is>
+      </c>
+      <c r="K45" s="15" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>Gouvêa, R.</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>Large devaluations and inflation inequality: Replicating Cravino and Levchenko (2017) with evidence from Brazil</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>Replicar Cravino-Levchenko (2017) con datos de Brasil para validar la robustez de los hallazgos en otro contexto LATAM.</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>Replicación metodológica con scanner data brasilera.</t>
+        </is>
+      </c>
+      <c r="H46" s="15" t="inlineStr">
+        <is>
+          <t>Los resultados de Cravino-Levchenko se replican en Brasil con magnitudes similares.</t>
+        </is>
+      </c>
+      <c r="I46" s="15" t="inlineStr">
+        <is>
+          <t>Antecedente LATAM de IPC distribuido durante devaluaciones. Refuerza la transferibilidad del marco al caso argentino.</t>
+        </is>
+      </c>
+      <c r="J46" s="15" t="inlineStr">
+        <is>
+          <t>https://onlinelibrary.wiley.com/doi/abs/10.1002/jae.2880</t>
+        </is>
+      </c>
+      <c r="K46" s="15" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>Del Canto, F., Grigsby, J., Qian, E., Walsh, C.</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>Are Inflationary Shocks Regressive? A Feasible Set Approach (NBER WP 31124)</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="F47" s="15" t="inlineStr">
+        <is>
+          <t>Medir el impacto distributivo de shocks inflacionarios a través del 'feasible set' (restricción presupuestaria + crédito).</t>
+        </is>
+      </c>
+      <c r="G47" s="15" t="inlineStr">
+        <is>
+          <t>Marco de feasible set + impulso-respuesta + microdatos de consumo, activos y trabajo por hogar.</t>
+        </is>
+      </c>
+      <c r="H47" s="15" t="inlineStr">
+        <is>
+          <t>Los shocks de oferta de petróleo son regresivos (golpean más a los pobres); los shocks de política monetaria expansiva son progresivos. El canal dominante es el efecto sobre precios de activos, no precios de bienes.</t>
+        </is>
+      </c>
+      <c r="I47" s="15" t="inlineStr">
+        <is>
+          <t>Marco reciente y técnicamente sofisticado. Cita en discusión cuando se interprete qué tipo de shock domina el período 2018-2025 en Argentina.</t>
+        </is>
+      </c>
+      <c r="J47" s="15" t="inlineStr">
+        <is>
+          <t>https://www.nber.org/papers/w31124</t>
+        </is>
+      </c>
+      <c r="K47" s="15" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>Kiss, R., Strasser, G.</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>Inflation Heterogeneity Across Households (ECB WP 2898)</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E48" s="15" t="inlineStr">
+        <is>
+          <t>WP</t>
+        </is>
+      </c>
+      <c r="F48" s="15" t="inlineStr">
+        <is>
+          <t>Estudiar la naturaleza, evolución y fuentes de la heterogeneidad de inflación entre hogares en Francia y Alemania.</t>
+        </is>
+      </c>
+      <c r="G48" s="15" t="inlineStr">
+        <is>
+          <t>Descomposición de la varianza de inflación por hogar entre componentes de precio y canasta.</t>
+        </is>
+      </c>
+      <c r="H48" s="15" t="inlineStr">
+        <is>
+          <t>Las diferencias de inflación entre hogares son grandes y persistentes. Las dos fuentes principales: diferencias espaciales en precios pagados por el MISMO producto + variedad específica del hogar dentro de categorías. El ingreso por sí solo no es un determinante relevante.</t>
+        </is>
+      </c>
+      <c r="I48" s="15" t="inlineStr">
+        <is>
+          <t>Replicación europea reciente del hallazgo de Kaplan-Schulhofer-Wohl. Refuerza la advertencia de que la heterogeneidad de canastas puede ser secundaria.</t>
+        </is>
+      </c>
+      <c r="J48" s="15" t="inlineStr">
+        <is>
+          <t>https://www.ecb.europa.eu/pub/pdf/scpwps/ecb.wp2898~29405f932f.en.pdf</t>
+        </is>
+      </c>
+      <c r="K48" s="15" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>Klick, J., Stockburger, A.</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>Examining U.S. inflation across households grouped by equivalized income (BLS Monthly Labor Review)</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>Económico</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>Nota técnica</t>
+        </is>
+      </c>
+      <c r="F49" s="15" t="inlineStr">
+        <is>
+          <t>Documentar la metodología BLS para construir IPCs por quintil de ingreso equivalizado.</t>
+        </is>
+      </c>
+      <c r="G49" s="15" t="inlineStr">
+        <is>
+          <t>Índices Laspeyres y Tornqvist Chained CPI-U por quintil; market basket shares biennial y monthly.</t>
+        </is>
+      </c>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>El quintil de ingresos más bajo tuvo 0.41 pp/año más de inflación que el más alto entre 2006-2022.</t>
+        </is>
+      </c>
+      <c r="I49" s="15" t="inlineStr">
+        <is>
+          <t>Referencia metodológica oficial BLS sobre construcción de D-CPI por subgrupo. Cita técnica para defender decisiones operativas.</t>
+        </is>
+      </c>
+      <c r="J49" s="15" t="inlineStr">
+        <is>
+          <t>https://www.bls.gov/opub/mlr/2024/article/examining-us-inflation-across-households-grouped-by-equivalized-income.htm</t>
+        </is>
+      </c>
+      <c r="K49" s="15" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>Alzuabi, R., Brown, S., Harris, M. N., Taylor, K.</t>
+        </is>
+      </c>
+      <c r="B50" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>Modelling the composition of household portfolios: A latent class approach</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Clustering microdata</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>Modelar la composición del portafolio de hogares (qué activos eligen) usando LCA sobre datos panel del UK Wealth and Assets Survey.</t>
+        </is>
+      </c>
+      <c r="G50" s="16" t="inlineStr">
+        <is>
+          <t>Latent Class Analysis con covariables sobre datos de hogares británicos.</t>
+        </is>
+      </c>
+      <c r="H50" s="16" t="inlineStr">
+        <is>
+          <t>Identifican subgrupos latentes de hogares con perfiles de portafolio distintos. La composición del portafolio se asocia con características demográficas y financieras.</t>
+        </is>
+      </c>
+      <c r="I50" s="16" t="inlineStr">
+        <is>
+          <t>Aplicación rigurosa de LCA a microdatos económicos de hogares (no a dietas/nutrición). Espejo metodológico cercano al pivote: clustering sobre comportamiento financiero del hogar.</t>
+        </is>
+      </c>
+      <c r="J50" s="16" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/caje.12691</t>
+        </is>
+      </c>
+      <c r="K50" s="16" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>Bénard, C., Näf, J., Josse, J.</t>
+        </is>
+      </c>
+      <c r="B51" s="17" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>MMD-based Variable Importance for Distributional Random Forest</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>Selección de variables</t>
+        </is>
+      </c>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F51" s="17" t="inlineStr">
+        <is>
+          <t>Proponer una medida de importancia de variables específica para Distributional Random Forests, basada en MMD (Maximum Mean Discrepancy) y el principio drop-and-relearn.</t>
+        </is>
+      </c>
+      <c r="G51" s="17" t="inlineStr">
+        <is>
+          <t>Algoritmo MMD + drop-and-relearn sobre DRF. Detecta variables que afectan la distribución completa, no solo la media.</t>
+        </is>
+      </c>
+      <c r="H51" s="17" t="inlineStr">
+        <is>
+          <t>Las medidas tradicionales (Sobol-MDA) detectan solo variables que afectan la media condicional; MMD detecta variables que afectan varianza, cuantiles o cualquier aspecto de la distribución. Outperforms competitors empíricamente.</t>
+        </is>
+      </c>
+      <c r="I51" s="17" t="inlineStr">
+        <is>
+          <t>Pieza CLAVE para el camino B (DRF): cómo seleccionar variables sociodemográficas para predecir el vector de shares. Cita técnica obligada si vas con DRF.</t>
+        </is>
+      </c>
+      <c r="J51" s="17" t="inlineStr">
+        <is>
+          <t>https://proceedings.mlr.press/v238/benard24a.html</t>
+        </is>
+      </c>
+      <c r="K51" s="17" t="inlineStr">
+        <is>
+          <t>TP — must-have ⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Lu, J., Shi, P., Li, H.</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Variable selection and inference strategies for multiple compositional regression</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>Selección de variables</t>
+        </is>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="inlineStr">
+        <is>
+          <t>Desarrollar y comparar estrategias de selección de variables (debiased lasso y resampling) en regresión lineal con covariables compositional.</t>
+        </is>
+      </c>
+      <c r="G52" s="17" t="inlineStr">
+        <is>
+          <t>Debiased lasso + bootstrap para intervalos de confianza válidos en regresiones compositional de alta dimensión.</t>
+        </is>
+      </c>
+      <c r="H52" s="17" t="inlineStr">
+        <is>
+          <t>Provee intervalos de confianza asintóticamente válidos para coeficientes individuales en regresión compositional, incluso con n pequeño.</t>
+        </is>
+      </c>
+      <c r="I52" s="17" t="inlineStr">
+        <is>
+          <t>Si se modela shares ~ sociodem (camino A) o se hace regresión compositional inversa, este es el método para seleccionar predictores. Geometría correcta para shares.</t>
+        </is>
+      </c>
+      <c r="J52" s="17" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/abs/pii/S0169743924000613</t>
+        </is>
+      </c>
+      <c r="K52" s="17" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>Susin, A., Wang, Y., Cao, K.-A., Calle, M. L.</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>Variable selection in microbiome compositional data analysis</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>Selección de variables</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>Paper (review)</t>
+        </is>
+      </c>
+      <c r="F53" s="17" t="inlineStr">
+        <is>
+          <t>Revisar y comparar métodos de selección de variables para datos compositional: selbal, clr-lasso, coda-lasso.</t>
+        </is>
+      </c>
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>Comparación empírica de tres familias de métodos para selección sparse en compositional data.</t>
+        </is>
+      </c>
+      <c r="H53" s="17" t="inlineStr">
+        <is>
+          <t>Cada método tiene fortalezas distintas: selbal (balances), clr-lasso (transformación), coda-lasso (penalización con suma cero). La elección depende de la densidad de la señal.</t>
+        </is>
+      </c>
+      <c r="I53" s="17" t="inlineStr">
+        <is>
+          <t>Aunque viene de microbiome, las técnicas son trasladables a shares de gasto (mismo problema: vector que suma 1, sparsity, compositional). Lectura en diagonal para elegir método.</t>
+        </is>
+      </c>
+      <c r="J53" s="17" t="inlineStr">
+        <is>
+          <t>https://academic.oup.com/nargab/article/2/2/lqaa029/5836692</t>
+        </is>
+      </c>
+      <c r="K53" s="17" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>Kursa, M. B., Rudnicki, W. R.</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>Feature Selection with the Boruta Package</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Selección de variables</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F54" s="17" t="inlineStr">
+        <is>
+          <t>Documentar el algoritmo Boruta para selección all-relevant de variables, basado en Random Forest + permuted shadow features.</t>
+        </is>
+      </c>
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>RF + shadow features (permutaciones aleatorias) + test estadístico iterativo para confirmar relevancia.</t>
+        </is>
+      </c>
+      <c r="H54" s="17" t="inlineStr">
+        <is>
+          <t>Boruta identifica todas las variables relevantes (no solo el subset mínimo). Maneja datos mixtos y no requiere asunciones distributivas.</t>
+        </is>
+      </c>
+      <c r="I54" s="17" t="inlineStr">
+        <is>
+          <t>Herramienta pragmática y plug-and-play. Si decidís camino B (DRF) o cualquier RF, Boruta es la primera vuelta de selección antes de Bénard-Näf-Josse.</t>
+        </is>
+      </c>
+      <c r="J54" s="17" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.18637/jss.v036.i11</t>
+        </is>
+      </c>
+      <c r="K54" s="17" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>Park, R., Choi, Y., Seo, M.</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>Lasso and Group Lasso with Categorical Predictors: Impact of Coding Strategy on Variable Selection and Prediction</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>Selección de variables</t>
+        </is>
+      </c>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="F55" s="17" t="inlineStr">
+        <is>
+          <t>Estudiar cómo la codificación de predictores categóricos (dummy, effect coding) afecta la selección y predicción en lasso y group lasso.</t>
+        </is>
+      </c>
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>Simulaciones + aplicación a MEPS (encuesta de salud).</t>
+        </is>
+      </c>
+      <c r="H55" s="17" t="inlineStr">
+        <is>
+          <t>Group lasso da selección consistente; la codificación importa para lasso pero no para regresión lineal sin penalización; group lasso tiende a sobre-incluir variables.</t>
+        </is>
+      </c>
+      <c r="I55" s="17" t="inlineStr">
+        <is>
+          <t>Si terminás haciendo regresión penalizada con sociodem (que son mayormente categóricas en EPH), este paper te ayuda a elegir codificación. Cita técnica para defender la decisión.</t>
+        </is>
+      </c>
+      <c r="J55" s="17" t="inlineStr">
+        <is>
+          <t>https://jbds.isdsa.org/jbds/article/view/64</t>
+        </is>
+      </c>
+      <c r="K55" s="17" t="inlineStr">
+        <is>
+          <t>TP — should-have</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K39"/>
+  <autoFilter ref="A1:K55"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>